<commit_message>
fix : excel to json window
파일을 선택해서 json이나 class로 변환할 수 있게 변경
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/EffectInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/EffectInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B96CCA6-89CF-4BCB-BA9D-480F9EF5F45E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE09ECD-3980-40B8-A490-91ECFC032466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17415" yWindow="4365" windowWidth="22965" windowHeight="11295" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="CSVEnums" sheetId="1" r:id="rId1"/>
@@ -70,10 +70,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>PhsycialDefence</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>MagicalDefence</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -98,15 +94,19 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>List&lt;Enum&lt;EffectType&gt;</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>hp회복</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>Hp</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>List&lt;Enum&lt;EffectType&gt;&gt;</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>PhysicalDefence</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1090,10 +1090,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1104,10 +1104,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1118,10 +1118,10 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1160,7 +1160,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -1174,7 +1174,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1185,10 +1185,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
feat : buff 기능 구현
</commit_message>
<xml_diff>
--- a/RPGProject/Assets/Project/Data/ExcelData/EffectInfo.xlsx
+++ b/RPGProject/Assets/Project/Data/ExcelData/EffectInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyb1\Documents\GitHub\RPG\RPGProject\Assets\Project\Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3223B2F-E492-408E-8B1E-9A5BECA3E1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DF73EE-AF9D-4A82-A0E7-C9B27CE07056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15855" yWindow="3240" windowWidth="14790" windowHeight="10695" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
+    <workbookView xWindow="4875" yWindow="3450" windowWidth="23220" windowHeight="10695" xr2:uid="{69A6533B-D580-4E18-8919-764171C47CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="CSVEnums" sheetId="1" r:id="rId1"/>

</xml_diff>